<commit_message>
feat(backlog): add dropdown Trạng thái 8 giá trị + cột Ghi chú
- Thêm cột Trạng thái (L) dạng dropdown 8 giá trị tiếng Việt qua hidden _Config sheet
- Thêm cột Ghi chú (N) với dữ liệu từ nguồn Backlog FPTvn & Roadmap 18.5
- Cập nhật Cover auto-formula cho đúng vị trí cột L (Trạng thái) và M (Nguồn)
- Color-coded format cho từng trạng thái; legend trực quan bên dưới bảng
- 31 tasks (18 BF + 13 RM), 14 cột A–N

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backlogpo/product_backlog_team.xlsx
+++ b/backlogpo/product_backlog_team.xlsx
@@ -7,16 +7,41 @@
     <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
-    <sheet name="📋 Cover" sheetId="1" r:id="rId1"/>
-    <sheet name="📌 Product Backlog" sheetId="2" r:id="rId2"/>
-    <sheet name="✅ Definition of Done" sheetId="3" r:id="rId3"/>
+    <sheet name="_Config" sheetId="1" r:id="rId1"/>
+    <sheet name="📋 Cover" sheetId="2" r:id="rId2"/>
+    <sheet name="📌 Product Backlog" sheetId="3" r:id="rId3"/>
+    <sheet name="✅ Definition of Done" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="283" uniqueCount="211">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="231">
+  <si>
+    <t>Chưa tiếp nhận yêu cầu</t>
+  </si>
+  <si>
+    <t>Đã tiếp nhận yêu cầu</t>
+  </si>
+  <si>
+    <t>Đang phân tích</t>
+  </si>
+  <si>
+    <t>Đang trao đổi PBLQ</t>
+  </si>
+  <si>
+    <t>Đã bàn giao ISC</t>
+  </si>
+  <si>
+    <t>In Progress DEV</t>
+  </si>
+  <si>
+    <t>UAT</t>
+  </si>
+  <si>
+    <t>Done</t>
+  </si>
   <si>
     <t>PRODUCT BACKLOG — FPT TELECOM</t>
   </si>
@@ -45,7 +70,7 @@
     <t>Ngày tạo</t>
   </si>
   <si>
-    <t>26/06/2026</t>
+    <t>28/06/2026</t>
   </si>
   <si>
     <t>Author</t>
@@ -57,34 +82,34 @@
     <t>Trạng thái</t>
   </si>
   <si>
-    <t>Draft v1.0</t>
+    <t>Draft v1.1</t>
   </si>
   <si>
     <t>Tổng Task Backlog</t>
   </si>
   <si>
-    <t>In Progress</t>
+    <t>Tổng SP</t>
   </si>
   <si>
     <t>Backlog FPTvn</t>
   </si>
   <si>
-    <t>To Do</t>
-  </si>
-  <si>
     <t>Roadmap 18.5</t>
   </si>
   <si>
-    <t>Chưa có Status</t>
-  </si>
-  <si>
-    <t>Tổng Story Points</t>
-  </si>
-  <si>
-    <t>High Priority</t>
-  </si>
-  <si>
-    <t>* Các ô màu cam tự động cập nhật khi thêm/sửa dữ liệu trong sheet Product Backlog.</t>
+    <t>Chưa tiếp nhận</t>
+  </si>
+  <si>
+    <t>Đã tiếp nhận</t>
+  </si>
+  <si>
+    <t>Đang phân tích / Trao đổi</t>
+  </si>
+  <si>
+    <t>Đã bàn giao ISC / DEV</t>
+  </si>
+  <si>
+    <t>* Các ô màu cam tự động cập nhật khi thêm/sửa dữ liệu. Cột Trạng thái có trình thả xuống — chọn từ danh sách 8 giai đoạn.</t>
   </si>
   <si>
     <t>PRODUCT BACKLOG — FPT TELECOM  |  FPT.vn &amp; HiFPT  |  Loại trừ: Done</t>
@@ -96,20 +121,24 @@
     <t>ID</t>
   </si>
   <si>
-    <t>Epic</t>
-  </si>
-  <si>
-    <t>Epic Name</t>
-  </si>
-  <si>
-    <t>US Title</t>
-  </si>
-  <si>
-    <t>User Story (thuần Việt)</t>
+    <t>Epic
+(để trống)</t>
+  </si>
+  <si>
+    <t>Epic Name
+(Sản phẩm)</t>
+  </si>
+  <si>
+    <t>US Title
+(Đầu mục công việc)</t>
+  </si>
+  <si>
+    <t>User Story
+(thuần Việt)</t>
   </si>
   <si>
     <t>Acceptance Criteria
-(Gherkin – CHO TRƯỚC/KHI/THÌ)</t>
+(CHO TRƯỚC / KHI / THÌ)</t>
   </si>
   <si>
     <t>SP</t>
@@ -127,10 +156,13 @@
 (BA)</t>
   </si>
   <si>
-    <t>Status</t>
+    <t>Trạng thái ▼</t>
   </si>
   <si>
     <t>Nguồn</t>
+  </si>
+  <si>
+    <t>Ghi chú</t>
   </si>
   <si>
     <t>BF-001</t>
@@ -151,6 +183,9 @@
   </si>
   <si>
     <t>15/04</t>
+  </si>
+  <si>
+    <t>Nhờ Hà check với chị Linh</t>
   </si>
   <si>
     <t>BF-002</t>
@@ -169,6 +204,9 @@
 THÌ dòng phí lắp đặt bị ẩn hoàn toàn</t>
   </si>
   <si>
+    <t>Đang làm việc với chính sách</t>
+  </si>
+  <si>
     <t>BF-003</t>
   </si>
   <si>
@@ -223,6 +261,9 @@
 THÌ điều hướng đúng đến luồng mua</t>
   </si>
   <si>
+    <t>22/5 golive 2 LDP</t>
+  </si>
+  <si>
     <t>BF-006</t>
   </si>
   <si>
@@ -272,6 +313,9 @@
 THÌ hệ thống yêu cầu xác thực email @fpt.com.vn
 KHI xác thực thành công
 THÌ hiển thị các gói cước ưu đãi dành riêng cho FPTers</t>
+  </si>
+  <si>
+    <t>Chờ FTQ phản hồi quy trình bán gói</t>
   </si>
   <si>
     <t>BF-009</t>
@@ -313,6 +357,9 @@
     <t>06/06/2026</t>
   </si>
   <si>
+    <t>Không ưu tiên giai đoạn này</t>
+  </si>
+  <si>
     <t>BF-011</t>
   </si>
   <si>
@@ -478,6 +525,9 @@
     <t>20/06</t>
   </si>
   <si>
+    <t>Chưa có chỗ nâng cấp camera combo trên HD net only</t>
+  </si>
+  <si>
     <t>RM-002</t>
   </si>
   <si>
@@ -497,6 +547,9 @@
     <t>06/03/2026</t>
   </si>
   <si>
+    <t>Cần làm rõ quy trình bán: chỉ sửa UI hay có luồng bán mới?</t>
+  </si>
+  <si>
     <t>RM-003</t>
   </si>
   <si>
@@ -576,6 +629,9 @@
 THÌ hệ thống tự trừ tiền và gửi thông báo; khi thất bại tôi nhận cảnh báo trong vòng 24 giờ</t>
   </si>
   <si>
+    <t>Cần làm rõ kịch bản thanh toán auto pay với team HiFPT</t>
+  </si>
+  <si>
     <t>RM-007</t>
   </si>
   <si>
@@ -595,6 +651,9 @@
 THÌ mã được ghi nhận và dịch vụ kích hoạt cho tài khoản họ</t>
   </si>
   <si>
+    <t>ISC đánh dấu KH đi theo luồng nhận mã; FPL trả thông tin qua ZNS</t>
+  </si>
+  <si>
     <t>RM-008</t>
   </si>
   <si>
@@ -611,6 +670,9 @@
 THÌ chuyển đúng đến luồng mua và chính sách được áp dụng đầy đủ</t>
   </si>
   <si>
+    <t>Cần đánh giá lại mức độ ưu tiên và xác nhận owner</t>
+  </si>
+  <si>
     <t>RM-009</t>
   </si>
   <si>
@@ -694,13 +756,16 @@
     <t>TỔNG</t>
   </si>
   <si>
-    <t>Chú thích ID:</t>
+    <t>Chú thích:</t>
   </si>
   <si>
     <t>BF-xxx = Backlog FPTvn</t>
   </si>
   <si>
     <t>RM-xxx = Roadmap 18.5</t>
+  </si>
+  <si>
+    <t>Cột L: Trạng thái có trình thả xuống — click ô để chọn</t>
   </si>
   <si>
     <t>Epic: để trống — PO/BA tự điền</t>
@@ -782,7 +847,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="21">
+  <fonts count="32">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -839,6 +904,13 @@
     </font>
     <font>
       <b/>
+      <sz val="10"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Times New Roman"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color rgb="FF1E4D8C"/>
       <name val="Times New Roman"/>
@@ -866,7 +938,8 @@
       <family val="2"/>
     </font>
     <font>
-      <sz val="11"/>
+      <b/>
+      <sz val="10"/>
       <color rgb="FF1E4D8C"/>
       <name val="Times New Roman"/>
       <family val="2"/>
@@ -879,14 +952,21 @@
       <family val="2"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FF5D4037"/>
+      <name val="Times New Roman"/>
+      <family val="2"/>
+    </font>
+    <font>
       <b/>
-      <sz val="11"/>
+      <sz val="10"/>
       <color rgb="FFE67E22"/>
       <name val="Times New Roman"/>
       <family val="2"/>
     </font>
     <font>
-      <sz val="11"/>
+      <b/>
+      <sz val="10"/>
       <color rgb="FFAAAAAA"/>
       <name val="Times New Roman"/>
       <family val="2"/>
@@ -915,7 +995,70 @@
     <font>
       <i/>
       <sz val="9"/>
+      <color rgb="FF555555"/>
+      <name val="Times New Roman"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="9"/>
       <color rgb="FF888888"/>
+      <name val="Times New Roman"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="8"/>
+      <color rgb="FFAAAAAA"/>
+      <name val="Times New Roman"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="8"/>
+      <color rgb="FF1E4D8C"/>
+      <name val="Times New Roman"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="8"/>
+      <color rgb="FF7D6608"/>
+      <name val="Times New Roman"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="8"/>
+      <color rgb="FF784212"/>
+      <name val="Times New Roman"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="8"/>
+      <color rgb="FF1A5276"/>
+      <name val="Times New Roman"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="8"/>
+      <color rgb="FFE67E22"/>
+      <name val="Times New Roman"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="8"/>
+      <color rgb="FF1E8449"/>
+      <name val="Times New Roman"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="8"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Times New Roman"/>
       <family val="2"/>
     </font>
@@ -926,7 +1069,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="19">
+  <fills count="24">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -965,13 +1108,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFAFAFA"/>
+        <fgColor rgb="FFF5F5F5"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFEF9E7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFDE7"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -989,13 +1138,25 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF0F5FF"/>
+        <fgColor rgb="FFEBEBEB"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFDF2E9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF3E0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF9C4"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1008,6 +1169,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFEBE0F5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFDEBD0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEAFAF1"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1078,7 +1251,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1102,85 +1275,121 @@
     <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="15" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="20" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="20" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="21" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="31" fillId="22" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="31" fillId="23" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1477,7 +1686,57 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A3:G17"/>
+  <dimension ref="A1:A8"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:1">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1">
+      <c r="A3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1">
+      <c r="A5" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1">
+      <c r="A6" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1">
+      <c r="A7" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1">
+      <c r="A8" t="s">
+        <v>7</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A3:G18"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="3.7109375" customWidth="1"/>
@@ -1486,7 +1745,7 @@
   <sheetData>
     <row r="3" spans="2:7" ht="50" customHeight="1">
       <c r="B3" s="1" t="s">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
@@ -1496,7 +1755,7 @@
     </row>
     <row r="4" spans="2:7" ht="30" customHeight="1">
       <c r="B4" s="2" t="s">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="C4" s="2"/>
       <c r="D4" s="2"/>
@@ -1514,55 +1773,55 @@
     </row>
     <row r="9" spans="2:7" ht="22" customHeight="1">
       <c r="B9" s="4" t="s">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="D9" s="5"/>
       <c r="E9" s="4" t="s">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="G9" s="5"/>
     </row>
     <row r="10" spans="2:7" ht="22" customHeight="1">
       <c r="B10" s="4" t="s">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="D10" s="5"/>
       <c r="E10" s="4" t="s">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="G10" s="5"/>
     </row>
     <row r="11" spans="2:7" ht="22" customHeight="1">
       <c r="B11" s="4" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="D11" s="5"/>
       <c r="E11" s="4" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="G11" s="5"/>
     </row>
     <row r="12" spans="2:7" ht="28" customHeight="1">
       <c r="B12" s="4" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="C12" s="6">
         <f>COUNTA('📌 Product Backlog'!A4:A34)</f>
@@ -1570,17 +1829,17 @@
       </c>
       <c r="D12" s="6"/>
       <c r="E12" s="4" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="F12" s="6">
-        <f>COUNTIF('📌 Product Backlog'!L4:L34,"In Progress")</f>
+        <f>SUM('📌 Product Backlog'!H4:H34)</f>
         <v>0</v>
       </c>
       <c r="G12" s="6"/>
     </row>
     <row r="13" spans="2:7" ht="28" customHeight="1">
       <c r="B13" s="4" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="C13" s="6">
         <f>COUNTIF('📌 Product Backlog'!M4:M34,"Backlog FPTvn")</f>
@@ -1588,62 +1847,80 @@
       </c>
       <c r="D13" s="6"/>
       <c r="E13" s="4" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="F13" s="6">
-        <f>COUNTIF('📌 Product Backlog'!L4:L34,"To Do")</f>
+        <f>COUNTIF('📌 Product Backlog'!M4:M34,"Roadmap 18.5")</f>
         <v>0</v>
       </c>
       <c r="G13" s="6"/>
     </row>
     <row r="14" spans="2:7" ht="28" customHeight="1">
       <c r="B14" s="4" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="C14" s="6">
-        <f>COUNTIF('📌 Product Backlog'!M4:M34,"Roadmap 18.5")</f>
+        <f>COUNTIF('📌 Product Backlog'!L4:L34,"Chưa tiếp nhận yêu cầu")</f>
         <v>0</v>
       </c>
       <c r="D14" s="6"/>
       <c r="E14" s="4" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="F14" s="6">
-        <f>COUNTBLANK('📌 Product Backlog'!L4:L34)</f>
+        <f>COUNTIF('📌 Product Backlog'!L4:L34,"Đã tiếp nhận yêu cầu")</f>
         <v>0</v>
       </c>
       <c r="G14" s="6"/>
     </row>
     <row r="15" spans="2:7" ht="28" customHeight="1">
       <c r="B15" s="4" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="C15" s="6">
-        <f>SUM('📌 Product Backlog'!H4:H34)</f>
+        <f>COUNTIF('📌 Product Backlog'!L4:L34,"Đang phân tích")+COUNTIF('📌 Product Backlog'!L4:L34,"Đang trao đổi PBLQ")</f>
         <v>0</v>
       </c>
       <c r="D15" s="6"/>
       <c r="E15" s="4" t="s">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="F15" s="6">
-        <f>COUNTIF('📌 Product Backlog'!G4:G34,"High")</f>
+        <f>COUNTIF('📌 Product Backlog'!L4:L34,"Đã bàn giao ISC")+COUNTIF('📌 Product Backlog'!L4:L34,"In Progress DEV")</f>
         <v>0</v>
       </c>
       <c r="G15" s="6"/>
     </row>
-    <row r="17" spans="2:7">
-      <c r="B17" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="C17" s="7"/>
-      <c r="D17" s="7"/>
-      <c r="E17" s="7"/>
-      <c r="F17" s="7"/>
-      <c r="G17" s="7"/>
+    <row r="16" spans="2:7" ht="28" customHeight="1">
+      <c r="B16" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C16" s="6">
+        <f>COUNTIF('📌 Product Backlog'!L4:L34,"UAT")</f>
+        <v>0</v>
+      </c>
+      <c r="D16" s="6"/>
+      <c r="E16" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="F16" s="6">
+        <f>COUNTIF('📌 Product Backlog'!L4:L34,"Done")</f>
+        <v>0</v>
+      </c>
+      <c r="G16" s="6"/>
+    </row>
+    <row r="18" spans="2:7">
+      <c r="B18" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="C18" s="7"/>
+      <c r="D18" s="7"/>
+      <c r="E18" s="7"/>
+      <c r="F18" s="7"/>
+      <c r="G18" s="7"/>
     </row>
   </sheetData>
-  <mergeCells count="18">
+  <mergeCells count="20">
     <mergeCell ref="B3:G3"/>
     <mergeCell ref="B4:G4"/>
     <mergeCell ref="B6:G6"/>
@@ -1661,15 +1938,17 @@
     <mergeCell ref="F14:G14"/>
     <mergeCell ref="C15:D15"/>
     <mergeCell ref="F15:G15"/>
-    <mergeCell ref="B17:G17"/>
+    <mergeCell ref="C16:D16"/>
+    <mergeCell ref="F16:G16"/>
+    <mergeCell ref="B18:G18"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M38"/>
+  <dimension ref="A1:N39"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="4.7109375" customWidth="1"/>
@@ -1677,17 +1956,18 @@
     <col min="3" max="3" width="6.7109375" customWidth="1"/>
     <col min="4" max="4" width="16.7109375" customWidth="1"/>
     <col min="5" max="5" width="22.7109375" customWidth="1"/>
-    <col min="6" max="7" width="34.7109375" customWidth="1"/>
+    <col min="6" max="7" width="33.7109375" customWidth="1"/>
     <col min="8" max="8" width="5.7109375" customWidth="1"/>
-    <col min="9" max="10" width="12.7109375" customWidth="1"/>
-    <col min="11" max="11" width="14.7109375" customWidth="1"/>
-    <col min="12" max="12" width="13.7109375" customWidth="1"/>
-    <col min="13" max="13" width="14.7109375" customWidth="1"/>
+    <col min="9" max="10" width="11.7109375" customWidth="1"/>
+    <col min="11" max="11" width="13.7109375" customWidth="1"/>
+    <col min="12" max="12" width="22.7109375" customWidth="1"/>
+    <col min="13" max="13" width="13.7109375" customWidth="1"/>
+    <col min="14" max="14" width="26.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="34" customHeight="1">
+    <row r="1" spans="1:14" ht="34" customHeight="1">
       <c r="A1" s="8" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="B1" s="8"/>
       <c r="C1" s="8"/>
@@ -1701,206 +1981,218 @@
       <c r="K1" s="8"/>
       <c r="L1" s="8"/>
       <c r="M1" s="8"/>
-    </row>
-    <row r="2" spans="1:13" ht="10" customHeight="1"/>
-    <row r="3" spans="1:13" ht="28" customHeight="1">
+      <c r="N1" s="8"/>
+    </row>
+    <row r="2" spans="1:14" ht="6" customHeight="1"/>
+    <row r="3" spans="1:14" ht="32" customHeight="1">
       <c r="A3" s="9" t="s">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="F3" s="9" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="G3" s="9" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="H3" s="9" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="I3" s="9" t="s">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="J3" s="9" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="K3" s="9" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="L3" s="9" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="M3" s="9" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13" ht="85" customHeight="1">
+        <v>44</v>
+      </c>
+      <c r="N3" s="9" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" ht="85" customHeight="1">
       <c r="A4" s="10">
         <v>1</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>37</v>
+        <v>46</v>
       </c>
       <c r="C4" s="12"/>
       <c r="D4" s="13" t="s">
-        <v>38</v>
+        <v>47</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="F4" s="13" t="s">
-        <v>40</v>
+        <v>49</v>
       </c>
       <c r="G4" s="13" t="s">
-        <v>41</v>
+        <v>50</v>
       </c>
       <c r="H4" s="15">
         <v>5</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="J4" s="10"/>
       <c r="K4" s="10"/>
       <c r="L4" s="16" t="s">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="M4" s="17" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" ht="85" customHeight="1">
-      <c r="A5" s="18">
+        <v>24</v>
+      </c>
+      <c r="N4" s="18" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" ht="85" customHeight="1">
+      <c r="A5" s="19">
         <v>2</v>
       </c>
-      <c r="B5" s="19" t="s">
-        <v>43</v>
-      </c>
-      <c r="C5" s="20"/>
-      <c r="D5" s="21" t="s">
-        <v>38</v>
-      </c>
-      <c r="E5" s="22" t="s">
-        <v>44</v>
-      </c>
-      <c r="F5" s="21" t="s">
-        <v>45</v>
-      </c>
-      <c r="G5" s="21" t="s">
-        <v>46</v>
-      </c>
-      <c r="H5" s="23">
+      <c r="B5" s="20" t="s">
+        <v>53</v>
+      </c>
+      <c r="C5" s="21"/>
+      <c r="D5" s="22" t="s">
+        <v>47</v>
+      </c>
+      <c r="E5" s="23" t="s">
+        <v>54</v>
+      </c>
+      <c r="F5" s="22" t="s">
+        <v>55</v>
+      </c>
+      <c r="G5" s="22" t="s">
+        <v>56</v>
+      </c>
+      <c r="H5" s="24">
         <v>5</v>
       </c>
-      <c r="I5" s="18" t="s">
-        <v>42</v>
-      </c>
-      <c r="J5" s="18"/>
-      <c r="K5" s="18"/>
-      <c r="L5" s="24" t="s">
-        <v>15</v>
+      <c r="I5" s="19" t="s">
+        <v>51</v>
+      </c>
+      <c r="J5" s="19"/>
+      <c r="K5" s="19"/>
+      <c r="L5" s="25" t="s">
+        <v>5</v>
       </c>
       <c r="M5" s="17" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13" ht="85" customHeight="1">
+        <v>24</v>
+      </c>
+      <c r="N5" s="26" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" ht="85" customHeight="1">
       <c r="A6" s="10">
         <v>3</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>47</v>
+        <v>58</v>
       </c>
       <c r="C6" s="12"/>
       <c r="D6" s="13" t="s">
-        <v>48</v>
+        <v>59</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>49</v>
+        <v>60</v>
       </c>
       <c r="F6" s="13" t="s">
-        <v>50</v>
+        <v>61</v>
       </c>
       <c r="G6" s="13" t="s">
-        <v>51</v>
+        <v>62</v>
       </c>
       <c r="H6" s="15">
         <v>5</v>
       </c>
       <c r="I6" s="10" t="s">
-        <v>52</v>
+        <v>63</v>
       </c>
       <c r="J6" s="10"/>
       <c r="K6" s="10"/>
       <c r="L6" s="16" t="s">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="M6" s="17" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13" ht="85" customHeight="1">
-      <c r="A7" s="18">
+        <v>24</v>
+      </c>
+      <c r="N6" s="18"/>
+    </row>
+    <row r="7" spans="1:14" ht="85" customHeight="1">
+      <c r="A7" s="19">
         <v>4</v>
       </c>
-      <c r="B7" s="19" t="s">
-        <v>53</v>
-      </c>
-      <c r="C7" s="20"/>
-      <c r="D7" s="21" t="s">
-        <v>48</v>
-      </c>
-      <c r="E7" s="22" t="s">
-        <v>54</v>
-      </c>
-      <c r="F7" s="21" t="s">
-        <v>55</v>
-      </c>
-      <c r="G7" s="21" t="s">
-        <v>56</v>
-      </c>
-      <c r="H7" s="23">
+      <c r="B7" s="20" t="s">
+        <v>64</v>
+      </c>
+      <c r="C7" s="21"/>
+      <c r="D7" s="22" t="s">
+        <v>59</v>
+      </c>
+      <c r="E7" s="23" t="s">
+        <v>65</v>
+      </c>
+      <c r="F7" s="22" t="s">
+        <v>66</v>
+      </c>
+      <c r="G7" s="22" t="s">
+        <v>67</v>
+      </c>
+      <c r="H7" s="24">
         <v>5</v>
       </c>
-      <c r="I7" s="18"/>
-      <c r="J7" s="18"/>
-      <c r="K7" s="18"/>
-      <c r="L7" s="24" t="s">
-        <v>15</v>
+      <c r="I7" s="19"/>
+      <c r="J7" s="19"/>
+      <c r="K7" s="19"/>
+      <c r="L7" s="25" t="s">
+        <v>5</v>
       </c>
       <c r="M7" s="17" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13" ht="85" customHeight="1">
+        <v>24</v>
+      </c>
+      <c r="N7" s="26"/>
+    </row>
+    <row r="8" spans="1:14" ht="85" customHeight="1">
       <c r="A8" s="10">
         <v>5</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>57</v>
+        <v>68</v>
       </c>
       <c r="C8" s="12"/>
       <c r="D8" s="13" t="s">
-        <v>48</v>
+        <v>59</v>
       </c>
       <c r="E8" s="14" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="F8" s="13" t="s">
-        <v>59</v>
+        <v>70</v>
       </c>
       <c r="G8" s="13" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="H8" s="15">
         <v>3</v>
@@ -1908,727 +2200,801 @@
       <c r="I8" s="10"/>
       <c r="J8" s="10"/>
       <c r="K8" s="10"/>
-      <c r="L8" s="24" t="s">
-        <v>15</v>
+      <c r="L8" s="25" t="s">
+        <v>5</v>
       </c>
       <c r="M8" s="17" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13" ht="85" customHeight="1">
-      <c r="A9" s="18">
+        <v>24</v>
+      </c>
+      <c r="N8" s="18" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" ht="85" customHeight="1">
+      <c r="A9" s="19">
         <v>6</v>
       </c>
-      <c r="B9" s="19" t="s">
-        <v>61</v>
-      </c>
-      <c r="C9" s="20"/>
-      <c r="D9" s="21"/>
-      <c r="E9" s="22" t="s">
-        <v>62</v>
-      </c>
-      <c r="F9" s="21" t="s">
-        <v>63</v>
-      </c>
-      <c r="G9" s="21" t="s">
-        <v>64</v>
-      </c>
-      <c r="H9" s="23">
+      <c r="B9" s="20" t="s">
+        <v>73</v>
+      </c>
+      <c r="C9" s="21"/>
+      <c r="D9" s="22"/>
+      <c r="E9" s="23" t="s">
+        <v>74</v>
+      </c>
+      <c r="F9" s="22" t="s">
+        <v>75</v>
+      </c>
+      <c r="G9" s="22" t="s">
+        <v>76</v>
+      </c>
+      <c r="H9" s="24">
         <v>5</v>
       </c>
-      <c r="I9" s="18"/>
-      <c r="J9" s="18"/>
-      <c r="K9" s="18"/>
-      <c r="L9" s="25"/>
+      <c r="I9" s="19"/>
+      <c r="J9" s="19"/>
+      <c r="K9" s="19"/>
+      <c r="L9" s="27" t="s">
+        <v>0</v>
+      </c>
       <c r="M9" s="17" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="10" spans="1:13" ht="85" customHeight="1">
+        <v>24</v>
+      </c>
+      <c r="N9" s="26"/>
+    </row>
+    <row r="10" spans="1:14" ht="85" customHeight="1">
       <c r="A10" s="10">
         <v>7</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>65</v>
+        <v>77</v>
       </c>
       <c r="C10" s="12"/>
       <c r="D10" s="13" t="s">
-        <v>38</v>
+        <v>47</v>
       </c>
       <c r="E10" s="14" t="s">
-        <v>66</v>
+        <v>78</v>
       </c>
       <c r="F10" s="13" t="s">
-        <v>67</v>
+        <v>79</v>
       </c>
       <c r="G10" s="13" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="H10" s="15">
         <v>5</v>
       </c>
       <c r="I10" s="10" t="s">
-        <v>69</v>
+        <v>81</v>
       </c>
       <c r="J10" s="10"/>
       <c r="K10" s="10"/>
-      <c r="L10" s="24" t="s">
-        <v>15</v>
+      <c r="L10" s="25" t="s">
+        <v>5</v>
       </c>
       <c r="M10" s="17" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="11" spans="1:13" ht="85" customHeight="1">
-      <c r="A11" s="18">
+        <v>24</v>
+      </c>
+      <c r="N10" s="18"/>
+    </row>
+    <row r="11" spans="1:14" ht="85" customHeight="1">
+      <c r="A11" s="19">
         <v>8</v>
       </c>
-      <c r="B11" s="19" t="s">
-        <v>70</v>
-      </c>
-      <c r="C11" s="20"/>
-      <c r="D11" s="21" t="s">
-        <v>48</v>
-      </c>
-      <c r="E11" s="22" t="s">
-        <v>71</v>
-      </c>
-      <c r="F11" s="21" t="s">
-        <v>72</v>
-      </c>
-      <c r="G11" s="21" t="s">
-        <v>73</v>
-      </c>
-      <c r="H11" s="23">
+      <c r="B11" s="20" t="s">
+        <v>82</v>
+      </c>
+      <c r="C11" s="21"/>
+      <c r="D11" s="22" t="s">
+        <v>59</v>
+      </c>
+      <c r="E11" s="23" t="s">
+        <v>83</v>
+      </c>
+      <c r="F11" s="22" t="s">
+        <v>84</v>
+      </c>
+      <c r="G11" s="22" t="s">
+        <v>85</v>
+      </c>
+      <c r="H11" s="24">
         <v>5</v>
       </c>
-      <c r="I11" s="18"/>
-      <c r="J11" s="18"/>
-      <c r="K11" s="18"/>
+      <c r="I11" s="19"/>
+      <c r="J11" s="19"/>
+      <c r="K11" s="19"/>
       <c r="L11" s="16" t="s">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="M11" s="17" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="12" spans="1:13" ht="85" customHeight="1">
+        <v>24</v>
+      </c>
+      <c r="N11" s="26" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" ht="85" customHeight="1">
       <c r="A12" s="10">
         <v>9</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>74</v>
+        <v>87</v>
       </c>
       <c r="C12" s="12"/>
       <c r="D12" s="13" t="s">
-        <v>38</v>
+        <v>47</v>
       </c>
       <c r="E12" s="14" t="s">
-        <v>75</v>
+        <v>88</v>
       </c>
       <c r="F12" s="13" t="s">
-        <v>76</v>
+        <v>89</v>
       </c>
       <c r="G12" s="13" t="s">
-        <v>77</v>
+        <v>90</v>
       </c>
       <c r="H12" s="15">
         <v>5</v>
       </c>
       <c r="I12" s="10" t="s">
-        <v>78</v>
+        <v>91</v>
       </c>
       <c r="J12" s="10"/>
       <c r="K12" s="10"/>
-      <c r="L12" s="25"/>
+      <c r="L12" s="27" t="s">
+        <v>0</v>
+      </c>
       <c r="M12" s="17" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="13" spans="1:13" ht="85" customHeight="1">
-      <c r="A13" s="18">
+        <v>24</v>
+      </c>
+      <c r="N12" s="18"/>
+    </row>
+    <row r="13" spans="1:14" ht="85" customHeight="1">
+      <c r="A13" s="19">
         <v>10</v>
       </c>
-      <c r="B13" s="19" t="s">
-        <v>79</v>
-      </c>
-      <c r="C13" s="20"/>
-      <c r="D13" s="21" t="s">
-        <v>48</v>
-      </c>
-      <c r="E13" s="22" t="s">
-        <v>80</v>
-      </c>
-      <c r="F13" s="21" t="s">
-        <v>81</v>
-      </c>
-      <c r="G13" s="21" t="s">
-        <v>82</v>
-      </c>
-      <c r="H13" s="23">
+      <c r="B13" s="20" t="s">
+        <v>92</v>
+      </c>
+      <c r="C13" s="21"/>
+      <c r="D13" s="22" t="s">
+        <v>59</v>
+      </c>
+      <c r="E13" s="23" t="s">
+        <v>93</v>
+      </c>
+      <c r="F13" s="22" t="s">
+        <v>94</v>
+      </c>
+      <c r="G13" s="22" t="s">
+        <v>95</v>
+      </c>
+      <c r="H13" s="24">
         <v>2</v>
       </c>
-      <c r="I13" s="18" t="s">
-        <v>83</v>
-      </c>
-      <c r="J13" s="18"/>
-      <c r="K13" s="18"/>
-      <c r="L13" s="25"/>
+      <c r="I13" s="19" t="s">
+        <v>96</v>
+      </c>
+      <c r="J13" s="19"/>
+      <c r="K13" s="19"/>
+      <c r="L13" s="27" t="s">
+        <v>0</v>
+      </c>
       <c r="M13" s="17" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="14" spans="1:13" ht="85" customHeight="1">
+        <v>24</v>
+      </c>
+      <c r="N13" s="26" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" ht="85" customHeight="1">
       <c r="A14" s="10">
         <v>11</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>84</v>
+        <v>98</v>
       </c>
       <c r="C14" s="12"/>
       <c r="D14" s="13" t="s">
-        <v>38</v>
+        <v>47</v>
       </c>
       <c r="E14" s="14" t="s">
-        <v>85</v>
+        <v>99</v>
       </c>
       <c r="F14" s="13" t="s">
-        <v>86</v>
+        <v>100</v>
       </c>
       <c r="G14" s="13" t="s">
-        <v>87</v>
+        <v>101</v>
       </c>
       <c r="H14" s="15">
         <v>3</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>88</v>
+        <v>102</v>
       </c>
       <c r="J14" s="10"/>
       <c r="K14" s="10"/>
-      <c r="L14" s="25"/>
+      <c r="L14" s="27" t="s">
+        <v>0</v>
+      </c>
       <c r="M14" s="17" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="15" spans="1:13" ht="85" customHeight="1">
-      <c r="A15" s="18">
+        <v>24</v>
+      </c>
+      <c r="N14" s="18"/>
+    </row>
+    <row r="15" spans="1:14" ht="85" customHeight="1">
+      <c r="A15" s="19">
         <v>12</v>
       </c>
-      <c r="B15" s="19" t="s">
-        <v>89</v>
-      </c>
-      <c r="C15" s="20"/>
-      <c r="D15" s="21" t="s">
-        <v>90</v>
-      </c>
-      <c r="E15" s="22" t="s">
-        <v>91</v>
-      </c>
-      <c r="F15" s="21" t="s">
-        <v>92</v>
-      </c>
-      <c r="G15" s="21" t="s">
-        <v>93</v>
-      </c>
-      <c r="H15" s="23">
+      <c r="B15" s="20" t="s">
+        <v>103</v>
+      </c>
+      <c r="C15" s="21"/>
+      <c r="D15" s="22" t="s">
+        <v>104</v>
+      </c>
+      <c r="E15" s="23" t="s">
+        <v>105</v>
+      </c>
+      <c r="F15" s="22" t="s">
+        <v>106</v>
+      </c>
+      <c r="G15" s="22" t="s">
+        <v>107</v>
+      </c>
+      <c r="H15" s="24">
         <v>2</v>
       </c>
-      <c r="I15" s="18" t="s">
-        <v>94</v>
-      </c>
-      <c r="J15" s="18"/>
-      <c r="K15" s="18"/>
-      <c r="L15" s="25"/>
+      <c r="I15" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="J15" s="19"/>
+      <c r="K15" s="19"/>
+      <c r="L15" s="27" t="s">
+        <v>0</v>
+      </c>
       <c r="M15" s="17" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="16" spans="1:13" ht="85" customHeight="1">
+        <v>24</v>
+      </c>
+      <c r="N15" s="26" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" ht="85" customHeight="1">
       <c r="A16" s="10">
         <v>13</v>
       </c>
       <c r="B16" s="11" t="s">
-        <v>95</v>
+        <v>109</v>
       </c>
       <c r="C16" s="12"/>
       <c r="D16" s="13" t="s">
-        <v>90</v>
+        <v>104</v>
       </c>
       <c r="E16" s="14" t="s">
-        <v>96</v>
+        <v>110</v>
       </c>
       <c r="F16" s="13" t="s">
-        <v>97</v>
+        <v>111</v>
       </c>
       <c r="G16" s="13" t="s">
-        <v>98</v>
+        <v>112</v>
       </c>
       <c r="H16" s="15">
         <v>3</v>
       </c>
       <c r="I16" s="10" t="s">
-        <v>99</v>
+        <v>113</v>
       </c>
       <c r="J16" s="10"/>
       <c r="K16" s="10"/>
-      <c r="L16" s="25"/>
+      <c r="L16" s="27" t="s">
+        <v>0</v>
+      </c>
       <c r="M16" s="17" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="17" spans="1:13" ht="85" customHeight="1">
-      <c r="A17" s="18">
+        <v>24</v>
+      </c>
+      <c r="N16" s="18"/>
+    </row>
+    <row r="17" spans="1:14" ht="85" customHeight="1">
+      <c r="A17" s="19">
         <v>14</v>
       </c>
-      <c r="B17" s="19" t="s">
-        <v>100</v>
-      </c>
-      <c r="C17" s="20"/>
-      <c r="D17" s="21" t="s">
-        <v>48</v>
-      </c>
-      <c r="E17" s="22" t="s">
-        <v>101</v>
-      </c>
-      <c r="F17" s="21" t="s">
-        <v>102</v>
-      </c>
-      <c r="G17" s="21" t="s">
-        <v>103</v>
-      </c>
-      <c r="H17" s="23">
+      <c r="B17" s="20" t="s">
+        <v>114</v>
+      </c>
+      <c r="C17" s="21"/>
+      <c r="D17" s="22" t="s">
+        <v>59</v>
+      </c>
+      <c r="E17" s="23" t="s">
+        <v>115</v>
+      </c>
+      <c r="F17" s="22" t="s">
+        <v>116</v>
+      </c>
+      <c r="G17" s="22" t="s">
+        <v>117</v>
+      </c>
+      <c r="H17" s="24">
         <v>5</v>
       </c>
-      <c r="I17" s="18" t="s">
-        <v>104</v>
-      </c>
-      <c r="J17" s="18"/>
-      <c r="K17" s="18"/>
-      <c r="L17" s="25"/>
+      <c r="I17" s="19" t="s">
+        <v>118</v>
+      </c>
+      <c r="J17" s="19"/>
+      <c r="K17" s="19"/>
+      <c r="L17" s="27" t="s">
+        <v>0</v>
+      </c>
       <c r="M17" s="17" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="18" spans="1:13" ht="85" customHeight="1">
+        <v>24</v>
+      </c>
+      <c r="N17" s="26"/>
+    </row>
+    <row r="18" spans="1:14" ht="85" customHeight="1">
       <c r="A18" s="10">
         <v>15</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>105</v>
+        <v>119</v>
       </c>
       <c r="C18" s="12"/>
       <c r="D18" s="13" t="s">
-        <v>48</v>
+        <v>59</v>
       </c>
       <c r="E18" s="14" t="s">
-        <v>106</v>
+        <v>120</v>
       </c>
       <c r="F18" s="13" t="s">
-        <v>107</v>
+        <v>121</v>
       </c>
       <c r="G18" s="13" t="s">
-        <v>108</v>
+        <v>122</v>
       </c>
       <c r="H18" s="15">
         <v>5</v>
       </c>
       <c r="I18" s="10" t="s">
-        <v>104</v>
+        <v>118</v>
       </c>
       <c r="J18" s="10"/>
       <c r="K18" s="10"/>
-      <c r="L18" s="25"/>
+      <c r="L18" s="27" t="s">
+        <v>0</v>
+      </c>
       <c r="M18" s="17" t="s">
+        <v>24</v>
+      </c>
+      <c r="N18" s="18"/>
+    </row>
+    <row r="19" spans="1:14" ht="85" customHeight="1">
+      <c r="A19" s="19">
         <v>16</v>
       </c>
-    </row>
-    <row r="19" spans="1:13" ht="85" customHeight="1">
-      <c r="A19" s="18">
-        <v>16</v>
-      </c>
-      <c r="B19" s="19" t="s">
-        <v>109</v>
-      </c>
-      <c r="C19" s="20"/>
-      <c r="D19" s="21" t="s">
-        <v>38</v>
-      </c>
-      <c r="E19" s="22" t="s">
-        <v>110</v>
-      </c>
-      <c r="F19" s="21" t="s">
-        <v>111</v>
-      </c>
-      <c r="G19" s="21" t="s">
-        <v>112</v>
-      </c>
-      <c r="H19" s="23">
+      <c r="B19" s="20" t="s">
+        <v>123</v>
+      </c>
+      <c r="C19" s="21"/>
+      <c r="D19" s="22" t="s">
+        <v>47</v>
+      </c>
+      <c r="E19" s="23" t="s">
+        <v>124</v>
+      </c>
+      <c r="F19" s="22" t="s">
+        <v>125</v>
+      </c>
+      <c r="G19" s="22" t="s">
+        <v>126</v>
+      </c>
+      <c r="H19" s="24">
         <v>5</v>
       </c>
-      <c r="I19" s="18" t="s">
-        <v>113</v>
-      </c>
-      <c r="J19" s="18"/>
-      <c r="K19" s="18"/>
-      <c r="L19" s="25"/>
+      <c r="I19" s="19" t="s">
+        <v>127</v>
+      </c>
+      <c r="J19" s="19"/>
+      <c r="K19" s="19"/>
+      <c r="L19" s="27" t="s">
+        <v>0</v>
+      </c>
       <c r="M19" s="17" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="20" spans="1:13" ht="85" customHeight="1">
+        <v>24</v>
+      </c>
+      <c r="N19" s="26"/>
+    </row>
+    <row r="20" spans="1:14" ht="85" customHeight="1">
       <c r="A20" s="10">
         <v>17</v>
       </c>
       <c r="B20" s="11" t="s">
-        <v>114</v>
+        <v>128</v>
       </c>
       <c r="C20" s="12"/>
       <c r="D20" s="13" t="s">
-        <v>38</v>
+        <v>47</v>
       </c>
       <c r="E20" s="14" t="s">
-        <v>115</v>
+        <v>129</v>
       </c>
       <c r="F20" s="13" t="s">
-        <v>116</v>
+        <v>130</v>
       </c>
       <c r="G20" s="13" t="s">
-        <v>117</v>
+        <v>131</v>
       </c>
       <c r="H20" s="15">
         <v>5</v>
       </c>
       <c r="I20" s="10" t="s">
-        <v>113</v>
+        <v>127</v>
       </c>
       <c r="J20" s="10"/>
       <c r="K20" s="10"/>
-      <c r="L20" s="25"/>
+      <c r="L20" s="27" t="s">
+        <v>0</v>
+      </c>
       <c r="M20" s="17" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="21" spans="1:13" ht="85" customHeight="1">
-      <c r="A21" s="18">
+        <v>24</v>
+      </c>
+      <c r="N20" s="18"/>
+    </row>
+    <row r="21" spans="1:14" ht="85" customHeight="1">
+      <c r="A21" s="19">
         <v>18</v>
       </c>
-      <c r="B21" s="19" t="s">
-        <v>118</v>
-      </c>
-      <c r="C21" s="20"/>
-      <c r="D21" s="21" t="s">
-        <v>38</v>
-      </c>
-      <c r="E21" s="22" t="s">
-        <v>119</v>
-      </c>
-      <c r="F21" s="21" t="s">
-        <v>120</v>
-      </c>
-      <c r="G21" s="21" t="s">
-        <v>121</v>
-      </c>
-      <c r="H21" s="23">
+      <c r="B21" s="20" t="s">
+        <v>132</v>
+      </c>
+      <c r="C21" s="21"/>
+      <c r="D21" s="22" t="s">
+        <v>47</v>
+      </c>
+      <c r="E21" s="23" t="s">
+        <v>133</v>
+      </c>
+      <c r="F21" s="22" t="s">
+        <v>134</v>
+      </c>
+      <c r="G21" s="22" t="s">
+        <v>135</v>
+      </c>
+      <c r="H21" s="24">
         <v>5</v>
       </c>
-      <c r="I21" s="18" t="s">
-        <v>113</v>
-      </c>
-      <c r="J21" s="18"/>
-      <c r="K21" s="18"/>
-      <c r="L21" s="25"/>
+      <c r="I21" s="19" t="s">
+        <v>127</v>
+      </c>
+      <c r="J21" s="19"/>
+      <c r="K21" s="19"/>
+      <c r="L21" s="27" t="s">
+        <v>0</v>
+      </c>
       <c r="M21" s="17" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="22" spans="1:13" ht="85" customHeight="1">
+        <v>24</v>
+      </c>
+      <c r="N21" s="26"/>
+    </row>
+    <row r="22" spans="1:14" ht="85" customHeight="1">
       <c r="A22" s="10">
         <v>19</v>
       </c>
-      <c r="B22" s="26" t="s">
-        <v>122</v>
+      <c r="B22" s="28" t="s">
+        <v>136</v>
       </c>
       <c r="C22" s="12"/>
       <c r="D22" s="13" t="s">
-        <v>38</v>
+        <v>47</v>
       </c>
       <c r="E22" s="14" t="s">
-        <v>123</v>
+        <v>137</v>
       </c>
       <c r="F22" s="13" t="s">
-        <v>124</v>
+        <v>138</v>
       </c>
       <c r="G22" s="13" t="s">
-        <v>125</v>
+        <v>139</v>
       </c>
       <c r="H22" s="15">
         <v>5</v>
       </c>
       <c r="I22" s="10" t="s">
-        <v>126</v>
+        <v>140</v>
       </c>
       <c r="J22" s="10"/>
       <c r="K22" s="10"/>
-      <c r="L22" s="24" t="s">
-        <v>15</v>
-      </c>
-      <c r="M22" s="27" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="23" spans="1:13" ht="85" customHeight="1">
-      <c r="A23" s="18">
+      <c r="L22" s="25" t="s">
+        <v>5</v>
+      </c>
+      <c r="M22" s="29" t="s">
+        <v>25</v>
+      </c>
+      <c r="N22" s="18" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="23" spans="1:14" ht="85" customHeight="1">
+      <c r="A23" s="19">
         <v>20</v>
       </c>
-      <c r="B23" s="28" t="s">
-        <v>127</v>
-      </c>
-      <c r="C23" s="20"/>
-      <c r="D23" s="21" t="s">
-        <v>48</v>
-      </c>
-      <c r="E23" s="22" t="s">
-        <v>128</v>
-      </c>
-      <c r="F23" s="21" t="s">
-        <v>129</v>
-      </c>
-      <c r="G23" s="21" t="s">
-        <v>130</v>
-      </c>
-      <c r="H23" s="23">
+      <c r="B23" s="30" t="s">
+        <v>142</v>
+      </c>
+      <c r="C23" s="21"/>
+      <c r="D23" s="22" t="s">
+        <v>59</v>
+      </c>
+      <c r="E23" s="23" t="s">
+        <v>143</v>
+      </c>
+      <c r="F23" s="22" t="s">
+        <v>144</v>
+      </c>
+      <c r="G23" s="22" t="s">
+        <v>145</v>
+      </c>
+      <c r="H23" s="24">
         <v>3</v>
       </c>
-      <c r="I23" s="18" t="s">
-        <v>131</v>
-      </c>
-      <c r="J23" s="18"/>
-      <c r="K23" s="18"/>
+      <c r="I23" s="19" t="s">
+        <v>146</v>
+      </c>
+      <c r="J23" s="19"/>
+      <c r="K23" s="19"/>
       <c r="L23" s="16" t="s">
-        <v>17</v>
-      </c>
-      <c r="M23" s="27" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="24" spans="1:13" ht="85" customHeight="1">
+        <v>1</v>
+      </c>
+      <c r="M23" s="29" t="s">
+        <v>25</v>
+      </c>
+      <c r="N23" s="26" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="24" spans="1:14" ht="85" customHeight="1">
       <c r="A24" s="10">
         <v>21</v>
       </c>
-      <c r="B24" s="26" t="s">
-        <v>132</v>
+      <c r="B24" s="28" t="s">
+        <v>148</v>
       </c>
       <c r="C24" s="12"/>
       <c r="D24" s="13" t="s">
-        <v>133</v>
+        <v>149</v>
       </c>
       <c r="E24" s="14" t="s">
-        <v>134</v>
+        <v>150</v>
       </c>
       <c r="F24" s="13" t="s">
-        <v>135</v>
+        <v>151</v>
       </c>
       <c r="G24" s="13" t="s">
-        <v>136</v>
+        <v>152</v>
       </c>
       <c r="H24" s="15">
         <v>3</v>
       </c>
       <c r="I24" s="10" t="s">
-        <v>137</v>
+        <v>153</v>
       </c>
       <c r="J24" s="10"/>
       <c r="K24" s="10"/>
-      <c r="L24" s="25"/>
-      <c r="M24" s="27" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="25" spans="1:13" ht="85" customHeight="1">
-      <c r="A25" s="18">
+      <c r="L24" s="27" t="s">
+        <v>0</v>
+      </c>
+      <c r="M24" s="29" t="s">
+        <v>25</v>
+      </c>
+      <c r="N24" s="18"/>
+    </row>
+    <row r="25" spans="1:14" ht="85" customHeight="1">
+      <c r="A25" s="19">
         <v>22</v>
       </c>
-      <c r="B25" s="28" t="s">
-        <v>138</v>
-      </c>
-      <c r="C25" s="20"/>
-      <c r="D25" s="21" t="s">
-        <v>139</v>
-      </c>
-      <c r="E25" s="22" t="s">
-        <v>140</v>
-      </c>
-      <c r="F25" s="21" t="s">
-        <v>141</v>
-      </c>
-      <c r="G25" s="21" t="s">
-        <v>142</v>
-      </c>
-      <c r="H25" s="23">
+      <c r="B25" s="30" t="s">
+        <v>154</v>
+      </c>
+      <c r="C25" s="21"/>
+      <c r="D25" s="22" t="s">
+        <v>155</v>
+      </c>
+      <c r="E25" s="23" t="s">
+        <v>156</v>
+      </c>
+      <c r="F25" s="22" t="s">
+        <v>157</v>
+      </c>
+      <c r="G25" s="22" t="s">
+        <v>158</v>
+      </c>
+      <c r="H25" s="24">
         <v>3</v>
       </c>
-      <c r="I25" s="18" t="s">
-        <v>137</v>
-      </c>
-      <c r="J25" s="18"/>
-      <c r="K25" s="18"/>
-      <c r="L25" s="25"/>
-      <c r="M25" s="27" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="26" spans="1:13" ht="85" customHeight="1">
+      <c r="I25" s="19" t="s">
+        <v>153</v>
+      </c>
+      <c r="J25" s="19"/>
+      <c r="K25" s="19"/>
+      <c r="L25" s="27" t="s">
+        <v>0</v>
+      </c>
+      <c r="M25" s="29" t="s">
+        <v>25</v>
+      </c>
+      <c r="N25" s="26"/>
+    </row>
+    <row r="26" spans="1:14" ht="85" customHeight="1">
       <c r="A26" s="10">
         <v>23</v>
       </c>
-      <c r="B26" s="26" t="s">
-        <v>143</v>
+      <c r="B26" s="28" t="s">
+        <v>159</v>
       </c>
       <c r="C26" s="12"/>
       <c r="D26" s="13" t="s">
-        <v>139</v>
+        <v>155</v>
       </c>
       <c r="E26" s="14" t="s">
-        <v>144</v>
+        <v>160</v>
       </c>
       <c r="F26" s="13" t="s">
-        <v>145</v>
+        <v>161</v>
       </c>
       <c r="G26" s="13" t="s">
-        <v>146</v>
+        <v>162</v>
       </c>
       <c r="H26" s="15">
         <v>3</v>
       </c>
       <c r="I26" s="10" t="s">
-        <v>147</v>
+        <v>163</v>
       </c>
       <c r="J26" s="10"/>
       <c r="K26" s="10"/>
-      <c r="L26" s="25"/>
-      <c r="M26" s="27" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="27" spans="1:13" ht="85" customHeight="1">
-      <c r="A27" s="18">
+      <c r="L26" s="27" t="s">
+        <v>0</v>
+      </c>
+      <c r="M26" s="29" t="s">
+        <v>25</v>
+      </c>
+      <c r="N26" s="18"/>
+    </row>
+    <row r="27" spans="1:14" ht="85" customHeight="1">
+      <c r="A27" s="19">
         <v>24</v>
       </c>
-      <c r="B27" s="28" t="s">
-        <v>148</v>
-      </c>
-      <c r="C27" s="20"/>
-      <c r="D27" s="21" t="s">
-        <v>149</v>
-      </c>
-      <c r="E27" s="22" t="s">
-        <v>150</v>
-      </c>
-      <c r="F27" s="21" t="s">
-        <v>151</v>
-      </c>
-      <c r="G27" s="21" t="s">
-        <v>152</v>
-      </c>
-      <c r="H27" s="23">
+      <c r="B27" s="30" t="s">
+        <v>164</v>
+      </c>
+      <c r="C27" s="21"/>
+      <c r="D27" s="22" t="s">
+        <v>165</v>
+      </c>
+      <c r="E27" s="23" t="s">
+        <v>166</v>
+      </c>
+      <c r="F27" s="22" t="s">
+        <v>167</v>
+      </c>
+      <c r="G27" s="22" t="s">
+        <v>168</v>
+      </c>
+      <c r="H27" s="24">
         <v>3</v>
       </c>
-      <c r="I27" s="18" t="s">
-        <v>137</v>
-      </c>
-      <c r="J27" s="18"/>
-      <c r="K27" s="18"/>
-      <c r="L27" s="25"/>
-      <c r="M27" s="27" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="28" spans="1:13" ht="85" customHeight="1">
+      <c r="I27" s="19" t="s">
+        <v>153</v>
+      </c>
+      <c r="J27" s="19"/>
+      <c r="K27" s="19"/>
+      <c r="L27" s="27" t="s">
+        <v>0</v>
+      </c>
+      <c r="M27" s="29" t="s">
+        <v>25</v>
+      </c>
+      <c r="N27" s="26" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="28" spans="1:14" ht="85" customHeight="1">
       <c r="A28" s="10">
         <v>25</v>
       </c>
-      <c r="B28" s="26" t="s">
-        <v>153</v>
+      <c r="B28" s="28" t="s">
+        <v>170</v>
       </c>
       <c r="C28" s="12"/>
       <c r="D28" s="13" t="s">
-        <v>154</v>
+        <v>171</v>
       </c>
       <c r="E28" s="14" t="s">
-        <v>155</v>
+        <v>172</v>
       </c>
       <c r="F28" s="13" t="s">
-        <v>156</v>
+        <v>173</v>
       </c>
       <c r="G28" s="13" t="s">
-        <v>157</v>
+        <v>174</v>
       </c>
       <c r="H28" s="15">
         <v>3</v>
       </c>
       <c r="I28" s="10" t="s">
-        <v>137</v>
+        <v>153</v>
       </c>
       <c r="J28" s="10"/>
       <c r="K28" s="10"/>
-      <c r="L28" s="25"/>
-      <c r="M28" s="27" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="29" spans="1:13" ht="85" customHeight="1">
-      <c r="A29" s="18">
+      <c r="L28" s="27" t="s">
+        <v>0</v>
+      </c>
+      <c r="M28" s="29" t="s">
+        <v>25</v>
+      </c>
+      <c r="N28" s="18" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="29" spans="1:14" ht="85" customHeight="1">
+      <c r="A29" s="19">
         <v>26</v>
       </c>
-      <c r="B29" s="28" t="s">
-        <v>158</v>
-      </c>
-      <c r="C29" s="20"/>
-      <c r="D29" s="21" t="s">
-        <v>38</v>
-      </c>
-      <c r="E29" s="22" t="s">
-        <v>159</v>
-      </c>
-      <c r="F29" s="21" t="s">
-        <v>160</v>
-      </c>
-      <c r="G29" s="21" t="s">
-        <v>161</v>
-      </c>
-      <c r="H29" s="23">
+      <c r="B29" s="30" t="s">
+        <v>176</v>
+      </c>
+      <c r="C29" s="21"/>
+      <c r="D29" s="22" t="s">
+        <v>47</v>
+      </c>
+      <c r="E29" s="23" t="s">
+        <v>177</v>
+      </c>
+      <c r="F29" s="22" t="s">
+        <v>178</v>
+      </c>
+      <c r="G29" s="22" t="s">
+        <v>179</v>
+      </c>
+      <c r="H29" s="24">
         <v>5</v>
       </c>
-      <c r="I29" s="18" t="s">
-        <v>137</v>
-      </c>
-      <c r="J29" s="18"/>
-      <c r="K29" s="18"/>
-      <c r="L29" s="25"/>
-      <c r="M29" s="27" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="30" spans="1:13" ht="85" customHeight="1">
+      <c r="I29" s="19" t="s">
+        <v>153</v>
+      </c>
+      <c r="J29" s="19"/>
+      <c r="K29" s="19"/>
+      <c r="L29" s="27" t="s">
+        <v>0</v>
+      </c>
+      <c r="M29" s="29" t="s">
+        <v>25</v>
+      </c>
+      <c r="N29" s="26" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="30" spans="1:14" ht="85" customHeight="1">
       <c r="A30" s="10">
         <v>27</v>
       </c>
-      <c r="B30" s="26" t="s">
-        <v>162</v>
+      <c r="B30" s="28" t="s">
+        <v>181</v>
       </c>
       <c r="C30" s="12"/>
       <c r="D30" s="13" t="s">
-        <v>48</v>
+        <v>59</v>
       </c>
       <c r="E30" s="14" t="s">
-        <v>163</v>
+        <v>182</v>
       </c>
       <c r="F30" s="13" t="s">
-        <v>164</v>
+        <v>183</v>
       </c>
       <c r="G30" s="13" t="s">
-        <v>165</v>
+        <v>184</v>
       </c>
       <c r="H30" s="15">
         <v>5</v>
@@ -2636,61 +3002,67 @@
       <c r="I30" s="10"/>
       <c r="J30" s="10"/>
       <c r="K30" s="10"/>
-      <c r="L30" s="25"/>
-      <c r="M30" s="27" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="31" spans="1:13" ht="85" customHeight="1">
-      <c r="A31" s="18">
+      <c r="L30" s="27" t="s">
+        <v>0</v>
+      </c>
+      <c r="M30" s="29" t="s">
+        <v>25</v>
+      </c>
+      <c r="N30" s="18"/>
+    </row>
+    <row r="31" spans="1:14" ht="85" customHeight="1">
+      <c r="A31" s="19">
         <v>28</v>
       </c>
-      <c r="B31" s="28" t="s">
-        <v>166</v>
-      </c>
-      <c r="C31" s="20"/>
-      <c r="D31" s="21" t="s">
-        <v>48</v>
-      </c>
-      <c r="E31" s="22" t="s">
-        <v>167</v>
-      </c>
-      <c r="F31" s="21" t="s">
-        <v>168</v>
-      </c>
-      <c r="G31" s="21" t="s">
-        <v>169</v>
-      </c>
-      <c r="H31" s="23">
+      <c r="B31" s="30" t="s">
+        <v>185</v>
+      </c>
+      <c r="C31" s="21"/>
+      <c r="D31" s="22" t="s">
+        <v>59</v>
+      </c>
+      <c r="E31" s="23" t="s">
+        <v>186</v>
+      </c>
+      <c r="F31" s="22" t="s">
+        <v>187</v>
+      </c>
+      <c r="G31" s="22" t="s">
+        <v>188</v>
+      </c>
+      <c r="H31" s="24">
         <v>5</v>
       </c>
-      <c r="I31" s="18"/>
-      <c r="J31" s="18"/>
-      <c r="K31" s="18"/>
-      <c r="L31" s="25"/>
-      <c r="M31" s="27" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="32" spans="1:13" ht="85" customHeight="1">
+      <c r="I31" s="19"/>
+      <c r="J31" s="19"/>
+      <c r="K31" s="19"/>
+      <c r="L31" s="27" t="s">
+        <v>0</v>
+      </c>
+      <c r="M31" s="29" t="s">
+        <v>25</v>
+      </c>
+      <c r="N31" s="26"/>
+    </row>
+    <row r="32" spans="1:14" ht="85" customHeight="1">
       <c r="A32" s="10">
         <v>29</v>
       </c>
-      <c r="B32" s="26" t="s">
-        <v>170</v>
+      <c r="B32" s="28" t="s">
+        <v>189</v>
       </c>
       <c r="C32" s="12"/>
       <c r="D32" s="13" t="s">
-        <v>90</v>
+        <v>104</v>
       </c>
       <c r="E32" s="14" t="s">
-        <v>171</v>
+        <v>190</v>
       </c>
       <c r="F32" s="13" t="s">
-        <v>172</v>
+        <v>191</v>
       </c>
       <c r="G32" s="13" t="s">
-        <v>173</v>
+        <v>192</v>
       </c>
       <c r="H32" s="15">
         <v>5</v>
@@ -2698,61 +3070,67 @@
       <c r="I32" s="10"/>
       <c r="J32" s="10"/>
       <c r="K32" s="10"/>
-      <c r="L32" s="25"/>
-      <c r="M32" s="27" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="33" spans="1:13" ht="85" customHeight="1">
-      <c r="A33" s="18">
+      <c r="L32" s="27" t="s">
+        <v>0</v>
+      </c>
+      <c r="M32" s="29" t="s">
+        <v>25</v>
+      </c>
+      <c r="N32" s="18"/>
+    </row>
+    <row r="33" spans="1:14" ht="85" customHeight="1">
+      <c r="A33" s="19">
         <v>30</v>
       </c>
-      <c r="B33" s="28" t="s">
-        <v>174</v>
-      </c>
-      <c r="C33" s="20"/>
-      <c r="D33" s="21" t="s">
-        <v>38</v>
-      </c>
-      <c r="E33" s="22" t="s">
-        <v>175</v>
-      </c>
-      <c r="F33" s="21" t="s">
-        <v>176</v>
-      </c>
-      <c r="G33" s="21" t="s">
-        <v>177</v>
-      </c>
-      <c r="H33" s="23">
+      <c r="B33" s="30" t="s">
+        <v>193</v>
+      </c>
+      <c r="C33" s="21"/>
+      <c r="D33" s="22" t="s">
+        <v>47</v>
+      </c>
+      <c r="E33" s="23" t="s">
+        <v>194</v>
+      </c>
+      <c r="F33" s="22" t="s">
+        <v>195</v>
+      </c>
+      <c r="G33" s="22" t="s">
+        <v>196</v>
+      </c>
+      <c r="H33" s="24">
         <v>5</v>
       </c>
-      <c r="I33" s="18"/>
-      <c r="J33" s="18"/>
-      <c r="K33" s="18"/>
-      <c r="L33" s="25"/>
-      <c r="M33" s="27" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="34" spans="1:13" ht="85" customHeight="1">
+      <c r="I33" s="19"/>
+      <c r="J33" s="19"/>
+      <c r="K33" s="19"/>
+      <c r="L33" s="27" t="s">
+        <v>0</v>
+      </c>
+      <c r="M33" s="29" t="s">
+        <v>25</v>
+      </c>
+      <c r="N33" s="26"/>
+    </row>
+    <row r="34" spans="1:14" ht="85" customHeight="1">
       <c r="A34" s="10">
         <v>31</v>
       </c>
-      <c r="B34" s="26" t="s">
-        <v>178</v>
+      <c r="B34" s="28" t="s">
+        <v>197</v>
       </c>
       <c r="C34" s="12"/>
       <c r="D34" s="13" t="s">
-        <v>38</v>
+        <v>47</v>
       </c>
       <c r="E34" s="14" t="s">
-        <v>179</v>
+        <v>198</v>
       </c>
       <c r="F34" s="13" t="s">
-        <v>180</v>
+        <v>199</v>
       </c>
       <c r="G34" s="13" t="s">
-        <v>181</v>
+        <v>200</v>
       </c>
       <c r="H34" s="15">
         <v>5</v>
@@ -2760,58 +3138,96 @@
       <c r="I34" s="10"/>
       <c r="J34" s="10"/>
       <c r="K34" s="10"/>
-      <c r="L34" s="25"/>
-      <c r="M34" s="27" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="36" spans="1:13" ht="24" customHeight="1">
-      <c r="A36" s="9" t="s">
-        <v>182</v>
-      </c>
-      <c r="B36" s="9"/>
-      <c r="C36" s="9"/>
-      <c r="D36" s="9"/>
-      <c r="E36" s="9"/>
-      <c r="F36" s="9"/>
-      <c r="G36" s="9"/>
-      <c r="H36" s="9">
+      <c r="L34" s="27" t="s">
+        <v>0</v>
+      </c>
+      <c r="M34" s="29" t="s">
+        <v>25</v>
+      </c>
+      <c r="N34" s="18"/>
+    </row>
+    <row r="36" spans="1:14" ht="24" customHeight="1">
+      <c r="A36" s="31" t="s">
+        <v>201</v>
+      </c>
+      <c r="B36" s="31"/>
+      <c r="C36" s="31"/>
+      <c r="D36" s="31"/>
+      <c r="E36" s="31"/>
+      <c r="F36" s="31"/>
+      <c r="G36" s="31"/>
+      <c r="H36" s="31">
         <f>SUM(H4:H34)</f>
         <v>0</v>
       </c>
-      <c r="I36" s="9">
+      <c r="I36" s="31">
         <f>COUNTA(A4:A34)&amp;" tasks"</f>
         <v>0</v>
       </c>
-      <c r="J36" s="9"/>
-      <c r="K36" s="9"/>
-      <c r="L36" s="9"/>
-      <c r="M36" s="9"/>
-    </row>
-    <row r="38" spans="1:13" ht="22" customHeight="1">
-      <c r="A38" s="29" t="s">
-        <v>183</v>
+      <c r="J36" s="31"/>
+      <c r="K36" s="31"/>
+      <c r="L36" s="31"/>
+      <c r="M36" s="31"/>
+      <c r="N36" s="31"/>
+    </row>
+    <row r="38" spans="1:14" ht="20" customHeight="1">
+      <c r="A38" s="32" t="s">
+        <v>202</v>
       </c>
       <c r="B38" s="17" t="s">
-        <v>184</v>
-      </c>
-      <c r="C38" s="27" t="s">
-        <v>185</v>
-      </c>
-      <c r="D38" s="30" t="s">
-        <v>186</v>
+        <v>203</v>
+      </c>
+      <c r="C38" s="29" t="s">
+        <v>204</v>
+      </c>
+      <c r="D38" s="33" t="s">
+        <v>205</v>
+      </c>
+      <c r="G38" s="34" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="39" spans="1:14" ht="18" customHeight="1">
+      <c r="A39" s="35" t="s">
+        <v>0</v>
+      </c>
+      <c r="B39" s="36" t="s">
+        <v>1</v>
+      </c>
+      <c r="C39" s="37" t="s">
+        <v>2</v>
+      </c>
+      <c r="D39" s="38" t="s">
+        <v>3</v>
+      </c>
+      <c r="E39" s="39" t="s">
+        <v>4</v>
+      </c>
+      <c r="F39" s="40" t="s">
+        <v>5</v>
+      </c>
+      <c r="G39" s="41" t="s">
+        <v>6</v>
+      </c>
+      <c r="H39" s="42" t="s">
+        <v>7</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:M1"/>
+    <mergeCell ref="A1:N1"/>
     <mergeCell ref="A36:G36"/>
   </mergeCells>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Giá trị không hợp lệ" error="Vui lòng chọn từ danh sách." promptTitle="Chọn trạng thái" prompt="Chưa tiếp nhận yêu cầu&#10;Đã tiếp nhận yêu cầu&#10;Đang phân tích&#10;Đang trao đổi PBLQ&#10;Đã bàn giao ISC&#10;In Progress DEV&#10;UAT&#10;Done" sqref="L4:L34">
+      <formula1>_Config!$A$1:$A$8</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C9"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -2823,97 +3239,97 @@
   <sheetData>
     <row r="1" spans="1:3" ht="30" customHeight="1">
       <c r="A1" s="8" t="s">
-        <v>187</v>
+        <v>207</v>
       </c>
       <c r="B1" s="8"/>
       <c r="C1" s="8"/>
     </row>
     <row r="2" spans="1:3" ht="22" customHeight="1">
       <c r="A2" s="9" t="s">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>188</v>
+        <v>208</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>189</v>
+        <v>209</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="26" customHeight="1">
-      <c r="A3" s="31" t="s">
-        <v>190</v>
-      </c>
-      <c r="B3" s="32" t="s">
-        <v>191</v>
-      </c>
-      <c r="C3" s="33" t="s">
-        <v>192</v>
+      <c r="A3" s="43" t="s">
+        <v>210</v>
+      </c>
+      <c r="B3" s="44" t="s">
+        <v>211</v>
+      </c>
+      <c r="C3" s="45" t="s">
+        <v>212</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="26" customHeight="1">
-      <c r="A4" s="31" t="s">
-        <v>193</v>
-      </c>
-      <c r="B4" s="34" t="s">
-        <v>194</v>
-      </c>
-      <c r="C4" s="35" t="s">
-        <v>195</v>
+      <c r="A4" s="43" t="s">
+        <v>213</v>
+      </c>
+      <c r="B4" s="46" t="s">
+        <v>214</v>
+      </c>
+      <c r="C4" s="47" t="s">
+        <v>215</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="26" customHeight="1">
-      <c r="A5" s="31" t="s">
-        <v>196</v>
-      </c>
-      <c r="B5" s="32" t="s">
-        <v>197</v>
-      </c>
-      <c r="C5" s="33" t="s">
-        <v>198</v>
+      <c r="A5" s="43" t="s">
+        <v>216</v>
+      </c>
+      <c r="B5" s="44" t="s">
+        <v>217</v>
+      </c>
+      <c r="C5" s="45" t="s">
+        <v>218</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="26" customHeight="1">
-      <c r="A6" s="31" t="s">
-        <v>199</v>
-      </c>
-      <c r="B6" s="34" t="s">
-        <v>200</v>
-      </c>
-      <c r="C6" s="35" t="s">
-        <v>201</v>
+      <c r="A6" s="43" t="s">
+        <v>219</v>
+      </c>
+      <c r="B6" s="46" t="s">
+        <v>220</v>
+      </c>
+      <c r="C6" s="47" t="s">
+        <v>221</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="26" customHeight="1">
-      <c r="A7" s="31" t="s">
-        <v>202</v>
-      </c>
-      <c r="B7" s="32" t="s">
-        <v>203</v>
-      </c>
-      <c r="C7" s="33" t="s">
-        <v>204</v>
+      <c r="A7" s="43" t="s">
+        <v>222</v>
+      </c>
+      <c r="B7" s="44" t="s">
+        <v>223</v>
+      </c>
+      <c r="C7" s="45" t="s">
+        <v>224</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="26" customHeight="1">
-      <c r="A8" s="31" t="s">
-        <v>205</v>
-      </c>
-      <c r="B8" s="34" t="s">
-        <v>206</v>
-      </c>
-      <c r="C8" s="35" t="s">
-        <v>207</v>
+      <c r="A8" s="43" t="s">
+        <v>225</v>
+      </c>
+      <c r="B8" s="46" t="s">
+        <v>226</v>
+      </c>
+      <c r="C8" s="47" t="s">
+        <v>227</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="26" customHeight="1">
-      <c r="A9" s="31" t="s">
-        <v>208</v>
-      </c>
-      <c r="B9" s="32" t="s">
-        <v>209</v>
-      </c>
-      <c r="C9" s="33" t="s">
-        <v>210</v>
+      <c r="A9" s="43" t="s">
+        <v>228</v>
+      </c>
+      <c r="B9" s="44" t="s">
+        <v>229</v>
+      </c>
+      <c r="C9" s="45" t="s">
+        <v>230</v>
       </c>
     </row>
   </sheetData>

</xml_diff>